<commit_message>
1.AI资源 - 切割动作 - 进入工程； 2. UI调整； 3. AI-mcp - 加入对 tilemap、animator、particle、timeline支持
</commit_message>
<xml_diff>
--- a/config/Config/Data/局内成长.xlsx
+++ b/config/Config/Data/局内成长.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="370">
   <si>
     <t>##var</t>
   </si>
@@ -609,13 +609,13 @@
     <t>event_industrial_shift</t>
   </si>
   <si>
-    <t>工业园又赶单</t>
-  </si>
-  <si>
-    <t>新项目落地，设备、资金、程序同时缺人。</t>
-  </si>
-  <si>
-    <t>线开起来了，下一波打得更狠。</t>
+    <t>网吧包夜还在赶单</t>
+  </si>
+  <si>
+    <t>包夜到一半，机房风扇罢工，进度条还在转。谁去接线？</t>
+  </si>
+  <si>
+    <t>线接上了，下一波开黑开得更狠。</t>
   </si>
   <si>
     <t>赶工出岔，全队被进度条抽了一下。</t>
@@ -624,10 +624,10 @@
     <t>event_leave_hometown</t>
   </si>
   <si>
-    <t>站台上各奔东西</t>
-  </si>
-  <si>
-    <t>有人上学，有人复读，有人先去打工。票根还热。</t>
+    <t>站台上先演离乡</t>
+  </si>
+  <si>
+    <t>分数没出，黄牛先走。有人上学，有人复读，有人去当网管。</t>
   </si>
   <si>
     <t>学霸把路线讲明白，随机兄弟更熟一分。</t>
@@ -636,19 +636,19 @@
     <t>AddAffinity</t>
   </si>
   <si>
-    <t>临走前先干一碗粉，大家回血。</t>
+    <t>票没抢到，先干一碗粉回血。</t>
   </si>
   <si>
     <t>event_hsr_construction</t>
   </si>
   <si>
-    <t>高铁工地催进度</t>
-  </si>
-  <si>
-    <t>桥隧和设备一起喊赶，安全帽满天飞。</t>
-  </si>
-  <si>
-    <t>施工组织顺了，下一波全队带盾。</t>
+    <t>光缆被挖，段位也掉</t>
+  </si>
+  <si>
+    <t>景观大道开挖，宿舍网先祭天。段位还在掉。</t>
+  </si>
+  <si>
+    <t>光缆接上了，下一波全队带盾。</t>
   </si>
   <si>
     <t>绕路赶场，全队被晒掉一层血。</t>
@@ -657,10 +657,10 @@
     <t>event_tourism_festival</t>
   </si>
   <si>
-    <t>围屋米酒摊开战</t>
-  </si>
-  <si>
-    <t>游客、米酒、舞台节目同时开场，摊主已经在喊人。</t>
+    <t>围屋空投先落地</t>
+  </si>
+  <si>
+    <t>空投砸在土楼顶上，米酒当急救包，摊主已经在喊人。</t>
   </si>
   <si>
     <t>Startup</t>
@@ -675,10 +675,10 @@
     <t>event_graduation_split</t>
   </si>
   <si>
-    <t>毕业季三岔口</t>
-  </si>
-  <si>
-    <t>工作、考研、考公三张表拍在桌上，先选哪个？</t>
+    <t>合同和志愿一起拍桌上</t>
+  </si>
+  <si>
+    <t>桌上三张纸：考研、考公、热爱游戏的加班合同。先点哪个？</t>
   </si>
   <si>
     <t>资料一共享，随机兄弟好感上涨。</t>
@@ -690,10 +690,10 @@
     <t>event_county_to_city</t>
   </si>
   <si>
-    <t>撤县设市的饼</t>
-  </si>
-  <si>
-    <t>建设、公服、商机一起涌来，窗口已经排到门口。</t>
+    <t>窗口排队领 404</t>
+  </si>
+  <si>
+    <t>窗口在发数字市民码，扫开 404。剪彩的横幅比服务器先到。</t>
   </si>
   <si>
     <t>Official</t>
@@ -708,10 +708,10 @@
     <t>event_return_home_tide</t>
   </si>
   <si>
-    <t>龙南东站人潮</t>
-  </si>
-  <si>
-    <t>高铁一停，过年回来的人把出站口堵成菜市场。</t>
+    <t>回村先给冰柜充值</t>
+  </si>
+  <si>
+    <t>人挤回来了。冰柜旁挂着充值，抢的是包间和充电宝。</t>
   </si>
   <si>
     <t>接站安排清楚，随机兄弟更熟。</t>
@@ -900,40 +900,40 @@
     <t>cohort_1997</t>
   </si>
   <si>
-    <t>97届兄弟出生年</t>
-  </si>
-  <si>
-    <t>这批兄弟大多出生于1997年前后。</t>
-  </si>
-  <si>
-    <t>作为共同纪年原点，不严格限制技能获得年份。</t>
+    <t>小卖部开始租卡带</t>
+  </si>
+  <si>
+    <t>97届还没站齐，柜台已经在数红白机卡带。通关的请辣条，没通的扫巷子。</t>
+  </si>
+  <si>
+    <t>共同纪年原点。波间当「从同一条巷子出门」，不卡就业技年份。</t>
   </si>
   <si>
     <t>Cohort</t>
   </si>
   <si>
-    <t>从同一座小城出发。</t>
-  </si>
-  <si>
-    <t>个人月份与年份可能前后浮动。</t>
+    <t>从同一座小城、同一台游戏机出发。</t>
+  </si>
+  <si>
+    <t>谁家先租到卡带，月份可以瞎编。</t>
   </si>
   <si>
     <t>Oral</t>
   </si>
   <si>
-    <t>兄弟口述</t>
+    <t>兄弟口述·卡带纪年</t>
   </si>
   <si>
     <t>economy_zone_2013</t>
   </si>
   <si>
-    <t>龙南经开区升级</t>
-  </si>
-  <si>
-    <t>2013年3月，龙南经开区升格为国家级经济技术开发区。</t>
-  </si>
-  <si>
-    <t>工业园订单、开发建设与就业机会同时增加。</t>
+    <t>工业园外开了通宵网吧</t>
+  </si>
+  <si>
+    <t>园里白班拧螺丝，园外通宵打页游。有人说这叫产业升级，有人说这叫包夜。</t>
+  </si>
+  <si>
+    <t>赶工单和开黑房同时进波间池。机械、互联网兄弟更容易撞见。</t>
   </si>
   <si>
     <t>Industry</t>
@@ -945,55 +945,58 @@
     <t>industrial_park</t>
   </si>
   <si>
-    <t>机械、互联网、银行、创业类兄弟更容易出现。</t>
-  </si>
-  <si>
-    <t>赶工、设备故障和经营风险同步增加。</t>
-  </si>
-  <si>
-    <t>龙南市人民政府·市情简介</t>
-  </si>
-  <si>
-    <t>http://www.jxln.gov.cn/lnzf/c103680/202308/f05e9c5bdbba43b1a65954a38ff99ac8.shtml</t>
+    <t>机械、互联网、银行、创业类更容易出现——有人接单，有人充点卡。</t>
+  </si>
+  <si>
+    <t>风扇一停，下一波怪会带着进度条冲过来。</t>
+  </si>
+  <si>
+    <t>Creative</t>
+  </si>
+  <si>
+    <t>玩法创作·网吧年鉴</t>
   </si>
   <si>
     <t>cohort_2015</t>
   </si>
   <si>
-    <t>2015毕业与离乡</t>
-  </si>
-  <si>
-    <t>多数兄弟于2015年前后高中毕业，升学或复读。</t>
-  </si>
-  <si>
-    <t>解锁大学、复读和提前就业的分流。</t>
+    <t>分数没出，火车票先黄了</t>
+  </si>
+  <si>
+    <t>高考刚完，站台已经在演「我去大城市做游戏」。分数线还在路上，行李已经过安检。</t>
+  </si>
+  <si>
+    <t>离乡分流：大学、复读、先去当网管。波间可遇外地同学。</t>
   </si>
   <si>
     <t>Education</t>
   </si>
   <si>
-    <t>Academic|Civil|Internet|Startup</t>
+    <t>Academic|Official|Internet|Startup</t>
   </si>
   <si>
     <t>station_home</t>
   </si>
   <si>
-    <t>同学关系延伸到不同学校和行业。</t>
-  </si>
-  <si>
-    <t>分隔异地，好感增长节奏变慢。</t>
+    <t>同学关系扩到不同机房和不同城市。</t>
+  </si>
+  <si>
+    <t>人已分开，好感长得慢。</t>
+  </si>
+  <si>
+    <t>兄弟口述·站台话</t>
   </si>
   <si>
     <t>hsr_build_2016</t>
   </si>
   <si>
-    <t>赣深高铁建设</t>
-  </si>
-  <si>
-    <t>2016年赣深高铁开工建设，龙南迎来高铁建设期。</t>
-  </si>
-  <si>
-    <t>工地、运输和设备事件增多。</t>
+    <t>景观大道把光缆挖断了</t>
+  </si>
+  <si>
+    <t>县城修景观大道，宿舍网先祭天。同一周王者开服，段位和路面一起翻修。</t>
+  </si>
+  <si>
+    <t>施工与掉线事件增多。土木、机械相遇加权。</t>
   </si>
   <si>
     <t>Transport</t>
@@ -1008,28 +1011,22 @@
     <t>土木与机械兄弟相遇概率提高。</t>
   </si>
   <si>
-    <t>施工期道路、噪声与赶工形成额外敌潮。</t>
-  </si>
-  <si>
-    <t>Media</t>
-  </si>
-  <si>
-    <t>龙南全域旅游与高铁建设报道</t>
-  </si>
-  <si>
-    <t>http://www.tourjie.com/article/1855.html</t>
+    <t>掉线和绕路一起上场，波次更挤。</t>
+  </si>
+  <si>
+    <t>玩法创作·断网纪年</t>
   </si>
   <si>
     <t>tourism_festival_2017</t>
   </si>
   <si>
-    <t>围美龙南旅游文化节</t>
-  </si>
-  <si>
-    <t>2017年起，龙南持续举办“围美龙南·客迎天下”旅游文化节。</t>
-  </si>
-  <si>
-    <t>围屋游客潮、米酒摊和舞台事件进入奖励池。</t>
+    <t>围屋被改成落地岛</t>
+  </si>
+  <si>
+    <t>游客还没到，吃鸡空投先到。米酒当急救包，土楼当盒子。</t>
+  </si>
+  <si>
+    <t>围屋游客潮、米酒救急包和空投事件进奖励池。</t>
   </si>
   <si>
     <t>Culture</t>
@@ -1041,28 +1038,25 @@
     <t>guanxi_wei</t>
   </si>
   <si>
-    <t>创业、烟草和学术类兄弟更易出现。</t>
-  </si>
-  <si>
-    <t>人潮、临时摊位和舞台事故提升波次密度。</t>
-  </si>
-  <si>
-    <t>中国江西网·围美龙南客迎天下</t>
-  </si>
-  <si>
-    <t>https://jxgz.jxnews.com.cn/system/2020/01/08/018717283.shtml</t>
+    <t>创业、烟草和学术类更易出现。</t>
+  </si>
+  <si>
+    <t>人潮、临时摊和成盒事故抬高波次密度。</t>
+  </si>
+  <si>
+    <t>玩法创作·成盒文化节</t>
   </si>
   <si>
     <t>graduation_2019</t>
   </si>
   <si>
-    <t>大学毕业与世客会申办</t>
-  </si>
-  <si>
-    <t>多数兄弟于2019年前后毕业；同年龙南获得第32届世客会举办权。</t>
-  </si>
-  <si>
-    <t>正式分流工作、考研、考公，并强化返乡联系。</t>
+    <t>第一份游戏民工合同</t>
+  </si>
+  <si>
+    <t>offer 写着热爱游戏，附件是无尽加班。有人考研，有人考公，有人点了同意并继续加班。</t>
+  </si>
+  <si>
+    <t>正式分流工作、考研、考公。波间见到带着 offer 的人。</t>
   </si>
   <si>
     <t>Academic|Official|Finance|Startup|Internet</t>
@@ -1071,25 +1065,22 @@
     <t>各行业兄弟开始带着就业技能回到队伍。</t>
   </si>
   <si>
-    <t>考试延期与求职失败会推迟就业技。</t>
-  </si>
-  <si>
-    <t>客家摇篮网·龙南获世客会承办权</t>
-  </si>
-  <si>
-    <t>http://www.gnhakka.com/n489/c196658/content.html</t>
+    <t>考试延期与求职失败仍会推迟就业技，大事件只改相遇。</t>
+  </si>
+  <si>
+    <t>玩法创作·合同纪年</t>
   </si>
   <si>
     <t>city_2020</t>
   </si>
   <si>
-    <t>龙南撤县设市</t>
-  </si>
-  <si>
-    <t>2020年6月，龙南撤县设市。</t>
-  </si>
-  <si>
-    <t>城市开发、公共服务和商业机会并存。</t>
+    <t>电竞一条街还在 PPT 里</t>
+  </si>
+  <si>
+    <t>广场剪了彩，服务器没到。窗口在发「数字市民」二维码，扫开是 404。</t>
+  </si>
+  <si>
+    <t>城市宣发与服务器没就绪并存。波间排窗口、扫码 404。</t>
   </si>
   <si>
     <t>Administrative</t>
@@ -1104,19 +1095,22 @@
     <t>开发、公职、银行与创业兄弟更容易相遇。</t>
   </si>
   <si>
-    <t>建设阵痛、岗位竞争和生活成本形成压力。</t>
+    <t>建设阵痛先到，岗位和生活成本变成波次压力。</t>
+  </si>
+  <si>
+    <t>玩法创作·PPT 广场</t>
   </si>
   <si>
     <t>hsr_open_2021</t>
   </si>
   <si>
-    <t>龙南进入高铁时代</t>
-  </si>
-  <si>
-    <t>2021年12月10日赣深高铁开通，龙南东站正式运营。</t>
-  </si>
-  <si>
-    <t>解锁龙南东站与返乡兄弟潮。</t>
+    <t>小卖部冰柜开始收点券</t>
+  </si>
+  <si>
+    <t>人从外地挤回来，柜台在冰棍旁边挂充值。抢的不是票，是包间和充电宝。</t>
+  </si>
+  <si>
+    <t>返乡潮进波间池。外地回来的兄弟更容易集合。</t>
   </si>
   <si>
     <t>Mechanical|Civil|Finance|Startup|Internet</t>
@@ -1125,16 +1119,13 @@
     <t>longnan_east</t>
   </si>
   <si>
-    <t>回乡过年和跨城工作的兄弟更容易重新集合。</t>
-  </si>
-  <si>
-    <t>客流高峰、抢票和接站混乱形成新敌潮。</t>
-  </si>
-  <si>
-    <t>龙南市人民政府·龙南东站正式运营</t>
-  </si>
-  <si>
-    <t>http://www.jxln.gov.cn/lnzf/c110699/202202/d5abc40cf11740a492181c764a313435.shtml</t>
+    <t>回乡过年和跨城加班的兄弟更容易重新集合。</t>
+  </si>
+  <si>
+    <t>抢的是包间和充电宝，人潮变成新敌潮。</t>
+  </si>
+  <si>
+    <t>玩法创作·点券冰柜</t>
   </si>
 </sst>
 </file>
@@ -1778,10 +1769,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD7"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2013,10 +2004,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD17"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2619,10 +2610,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD15"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2902,7 +2893,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>196</v>
       </c>
@@ -2934,7 +2925,7 @@
         <v>0.07</v>
       </c>
     </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>201</v>
       </c>
@@ -2966,7 +2957,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>207</v>
       </c>
@@ -2998,7 +2989,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>212</v>
       </c>
@@ -3030,7 +3021,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>218</v>
       </c>
@@ -3062,7 +3053,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>223</v>
       </c>
@@ -3094,7 +3085,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>229</v>
       </c>
@@ -3794,16 +3785,16 @@
         <v>310</v>
       </c>
       <c r="Q5" t="s">
-        <v>226</v>
+        <v>311</v>
       </c>
       <c r="R5" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="S5" t="s">
-        <v>312</v>
+        <v>24</v>
       </c>
       <c r="T5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
@@ -3859,7 +3850,7 @@
         <v>300</v>
       </c>
       <c r="R6" t="s">
-        <v>301</v>
+        <v>322</v>
       </c>
       <c r="S6" t="s">
         <v>24</v>
@@ -3873,7 +3864,7 @@
         <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C7">
         <v>2016</v>
@@ -3882,13 +3873,13 @@
         <v>30</v>
       </c>
       <c r="E7" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F7" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="G7" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="H7" t="s">
         <v>31</v>
@@ -3897,10 +3888,10 @@
         <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="K7" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="L7">
         <v>2</v>
@@ -3909,25 +3900,25 @@
         <v>207</v>
       </c>
       <c r="N7" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="O7" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="P7" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="Q7" t="s">
-        <v>331</v>
+        <v>311</v>
       </c>
       <c r="R7" t="s">
         <v>332</v>
       </c>
       <c r="S7" t="s">
-        <v>333</v>
+        <v>24</v>
       </c>
       <c r="T7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
@@ -3935,7 +3926,7 @@
         <v>24</v>
       </c>
       <c r="B8" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C8">
         <v>2017</v>
@@ -3944,13 +3935,13 @@
         <v>40</v>
       </c>
       <c r="E8" t="s">
+        <v>334</v>
+      </c>
+      <c r="F8" t="s">
         <v>335</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>336</v>
-      </c>
-      <c r="G8" t="s">
-        <v>337</v>
       </c>
       <c r="H8" t="s">
         <v>31</v>
@@ -3959,10 +3950,10 @@
         <v>1</v>
       </c>
       <c r="J8" t="s">
+        <v>337</v>
+      </c>
+      <c r="K8" t="s">
         <v>338</v>
-      </c>
-      <c r="K8" t="s">
-        <v>339</v>
       </c>
       <c r="L8">
         <v>1.7</v>
@@ -3971,25 +3962,25 @@
         <v>212</v>
       </c>
       <c r="N8" t="s">
+        <v>339</v>
+      </c>
+      <c r="O8" t="s">
         <v>340</v>
       </c>
-      <c r="O8" t="s">
+      <c r="P8" t="s">
         <v>341</v>
       </c>
-      <c r="P8" t="s">
+      <c r="Q8" t="s">
+        <v>311</v>
+      </c>
+      <c r="R8" t="s">
         <v>342</v>
       </c>
-      <c r="Q8" t="s">
-        <v>331</v>
-      </c>
-      <c r="R8" t="s">
-        <v>343</v>
-      </c>
       <c r="S8" t="s">
-        <v>344</v>
+        <v>24</v>
       </c>
       <c r="T8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
@@ -3997,7 +3988,7 @@
         <v>24</v>
       </c>
       <c r="B9" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="C9">
         <v>2019</v>
@@ -4006,13 +3997,13 @@
         <v>50</v>
       </c>
       <c r="E9" t="s">
+        <v>344</v>
+      </c>
+      <c r="F9" t="s">
+        <v>345</v>
+      </c>
+      <c r="G9" t="s">
         <v>346</v>
-      </c>
-      <c r="F9" t="s">
-        <v>347</v>
-      </c>
-      <c r="G9" t="s">
-        <v>348</v>
       </c>
       <c r="H9" t="s">
         <v>33</v>
@@ -4024,7 +4015,7 @@
         <v>317</v>
       </c>
       <c r="K9" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="L9">
         <v>1.9</v>
@@ -4036,22 +4027,22 @@
         <v>319</v>
       </c>
       <c r="O9" t="s">
+        <v>348</v>
+      </c>
+      <c r="P9" t="s">
+        <v>349</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>311</v>
+      </c>
+      <c r="R9" t="s">
         <v>350</v>
       </c>
-      <c r="P9" t="s">
-        <v>351</v>
-      </c>
-      <c r="Q9" t="s">
-        <v>331</v>
-      </c>
-      <c r="R9" t="s">
-        <v>352</v>
-      </c>
       <c r="S9" t="s">
-        <v>353</v>
+        <v>24</v>
       </c>
       <c r="T9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
@@ -4059,7 +4050,7 @@
         <v>24</v>
       </c>
       <c r="B10" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="C10">
         <v>2020</v>
@@ -4068,13 +4059,13 @@
         <v>60</v>
       </c>
       <c r="E10" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="F10" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="G10" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="H10" t="s">
         <v>33</v>
@@ -4083,10 +4074,10 @@
         <v>1</v>
       </c>
       <c r="J10" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="K10" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="L10">
         <v>1.8</v>
@@ -4095,25 +4086,25 @@
         <v>223</v>
       </c>
       <c r="N10" t="s">
+        <v>357</v>
+      </c>
+      <c r="O10" t="s">
+        <v>358</v>
+      </c>
+      <c r="P10" t="s">
+        <v>359</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>311</v>
+      </c>
+      <c r="R10" t="s">
         <v>360</v>
       </c>
-      <c r="O10" t="s">
-        <v>361</v>
-      </c>
-      <c r="P10" t="s">
-        <v>362</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>226</v>
-      </c>
-      <c r="R10" t="s">
-        <v>311</v>
-      </c>
       <c r="S10" t="s">
-        <v>312</v>
+        <v>24</v>
       </c>
       <c r="T10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
@@ -4121,7 +4112,7 @@
         <v>24</v>
       </c>
       <c r="B11" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="C11">
         <v>2021</v>
@@ -4130,13 +4121,13 @@
         <v>70</v>
       </c>
       <c r="E11" t="s">
+        <v>362</v>
+      </c>
+      <c r="F11" t="s">
+        <v>363</v>
+      </c>
+      <c r="G11" t="s">
         <v>364</v>
-      </c>
-      <c r="F11" t="s">
-        <v>365</v>
-      </c>
-      <c r="G11" t="s">
-        <v>366</v>
       </c>
       <c r="H11" t="s">
         <v>33</v>
@@ -4145,10 +4136,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="K11" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="L11">
         <v>2</v>
@@ -4157,25 +4148,25 @@
         <v>229</v>
       </c>
       <c r="N11" t="s">
+        <v>366</v>
+      </c>
+      <c r="O11" t="s">
+        <v>367</v>
+      </c>
+      <c r="P11" t="s">
         <v>368</v>
       </c>
-      <c r="O11" t="s">
+      <c r="Q11" t="s">
+        <v>311</v>
+      </c>
+      <c r="R11" t="s">
         <v>369</v>
       </c>
-      <c r="P11" t="s">
-        <v>370</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>226</v>
-      </c>
-      <c r="R11" t="s">
-        <v>371</v>
-      </c>
       <c r="S11" t="s">
-        <v>372</v>
+        <v>24</v>
       </c>
       <c r="T11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>